<commit_message>
May 20, 2026, 5:46 PM
</commit_message>
<xml_diff>
--- a/storage/exports/4/07TCRPS8655B1ZK/022026/gstr1.xlsx
+++ b/storage/exports/4/07TCRPS8655B1ZK/022026/gstr1.xlsx
@@ -1121,7 +1121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelRow="0"/>
   <cols>
     <col width="50.7109375" customWidth="1" min="1" max="1"/>
@@ -1207,16 +1207,16 @@
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>FAWRLX2600000063</t>
+          <t>6p5kc26102</t>
         </is>
       </c>
       <c r="C5" s="0" t="inlineStr">
         <is>
-          <t>FAWRLX2600000079</t>
+          <t>6p5kc26132</t>
         </is>
       </c>
       <c r="D5" s="0" t="n">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="E5" s="0" t="n">
         <v>0</v>
@@ -1230,16 +1230,16 @@
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>RAT6SO2600000021</t>
+          <t>6p5kc26C50</t>
         </is>
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
-          <t>RAT6SO2600000027</t>
+          <t>6p5kc26C65</t>
         </is>
       </c>
       <c r="D6" s="0" t="n">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E6" s="0" t="n">
         <v>0</v>
@@ -1248,21 +1248,21 @@
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t>Credit Note</t>
+          <t>Invoices for outward supply</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>CANQ1W2600000008</t>
+          <t>IN-4</t>
         </is>
       </c>
       <c r="C7" s="0" t="inlineStr">
         <is>
-          <t>CANQ1W2600000012</t>
+          <t>IN-4</t>
         </is>
       </c>
       <c r="D7" s="0" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E7" s="0" t="n">
         <v>0</v>
@@ -1271,23 +1271,92 @@
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
+          <t>Invoices for outward supply</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>FAWRLX2600000063</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>FAWRLX2600000079</t>
+        </is>
+      </c>
+      <c r="D8" s="0" t="n">
+        <v>17</v>
+      </c>
+      <c r="E8" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>Credit Note</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>RAT6SO2600000021</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>RAT6SO2600000027</t>
+        </is>
+      </c>
+      <c r="D9" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="E9" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>Credit Note</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>CANQ1W2600000008</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>CANQ1W2600000012</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
           <t>Debit Note</t>
         </is>
       </c>
-      <c r="B8" s="0" t="inlineStr">
+      <c r="B11" s="0" t="inlineStr">
         <is>
           <t>DAL84U2600000004</t>
         </is>
       </c>
-      <c r="C8" s="0" t="inlineStr">
+      <c r="C11" s="0" t="inlineStr">
         <is>
           <t>DAL84U2600000004</t>
         </is>
       </c>
-      <c r="D8" s="0" t="n">
+      <c r="D11" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="0" t="n">
+      <c r="E11" s="0" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1451,7 +1520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelRow="0"/>
   <cols>
     <col width="22.42578125" customWidth="1" min="1" max="1"/>
@@ -1563,7 +1632,7 @@
         <v>3</v>
       </c>
       <c r="E5" s="0" t="n">
-        <v>90.29000000000001</v>
+        <v>578.64</v>
       </c>
       <c r="F5" s="0" t="n">
         <v>0</v>
@@ -1665,7 +1734,7 @@
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>06-Haryana</t>
+          <t>07-Delhi</t>
         </is>
       </c>
       <c r="C10" s="0" t="n"/>
@@ -1673,7 +1742,7 @@
         <v>3</v>
       </c>
       <c r="E10" s="0" t="n">
-        <v>0</v>
+        <v>516.5</v>
       </c>
       <c r="F10" s="0" t="n">
         <v>0</v>
@@ -1687,7 +1756,7 @@
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>20-Jharkhand</t>
+          <t>24-Gujarat</t>
         </is>
       </c>
       <c r="C11" s="0" t="n"/>
@@ -1695,7 +1764,7 @@
         <v>3</v>
       </c>
       <c r="E11" s="0" t="n">
-        <v>0</v>
+        <v>219.42</v>
       </c>
       <c r="F11" s="0" t="n">
         <v>0</v>
@@ -1709,7 +1778,7 @@
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>29-Karnataka</t>
+          <t>06-Haryana</t>
         </is>
       </c>
       <c r="C12" s="0" t="n"/>
@@ -1717,7 +1786,7 @@
         <v>3</v>
       </c>
       <c r="E12" s="0" t="n">
-        <v>318.46</v>
+        <v>0</v>
       </c>
       <c r="F12" s="0" t="n">
         <v>0</v>
@@ -1731,7 +1800,7 @@
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>27-Maharashtra</t>
+          <t>02-Himachal Pradesh</t>
         </is>
       </c>
       <c r="C13" s="0" t="n"/>
@@ -1739,7 +1808,7 @@
         <v>3</v>
       </c>
       <c r="E13" s="0" t="n">
-        <v>126.21</v>
+        <v>200</v>
       </c>
       <c r="F13" s="0" t="n">
         <v>0</v>
@@ -1753,7 +1822,7 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>03-Punjab</t>
+          <t>20-Jharkhand</t>
         </is>
       </c>
       <c r="C14" s="0" t="n"/>
@@ -1761,7 +1830,7 @@
         <v>3</v>
       </c>
       <c r="E14" s="0" t="n">
-        <v>111.66</v>
+        <v>0</v>
       </c>
       <c r="F14" s="0" t="n">
         <v>0</v>
@@ -1775,7 +1844,7 @@
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>33-Tamil Nadu</t>
+          <t>29-Karnataka</t>
         </is>
       </c>
       <c r="C15" s="0" t="n"/>
@@ -1783,7 +1852,7 @@
         <v>3</v>
       </c>
       <c r="E15" s="0" t="n">
-        <v>113.59</v>
+        <v>654.38</v>
       </c>
       <c r="F15" s="0" t="n">
         <v>0</v>
@@ -1797,7 +1866,7 @@
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>36-Telangana</t>
+          <t>27-Maharashtra</t>
         </is>
       </c>
       <c r="C16" s="0" t="n"/>
@@ -1805,7 +1874,7 @@
         <v>3</v>
       </c>
       <c r="E16" s="0" t="n">
-        <v>0</v>
+        <v>319.41</v>
       </c>
       <c r="F16" s="0" t="n">
         <v>0</v>
@@ -1819,7 +1888,7 @@
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>19-West Bengal</t>
+          <t>21-Odisha</t>
         </is>
       </c>
       <c r="C17" s="0" t="n"/>
@@ -1830,6 +1899,116 @@
         <v>0</v>
       </c>
       <c r="F17" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>03-Punjab</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="n"/>
+      <c r="D18" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" s="0" t="n">
+        <v>315.54</v>
+      </c>
+      <c r="F18" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>08-Rajasthan</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="n"/>
+      <c r="D19" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" s="0" t="n">
+        <v>113.59</v>
+      </c>
+      <c r="F19" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>33-Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="n"/>
+      <c r="D20" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" s="0" t="n">
+        <v>524.27</v>
+      </c>
+      <c r="F20" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="inlineStr">
+        <is>
+          <t>19-West Bengal</t>
+        </is>
+      </c>
+      <c r="C21" s="0" t="n"/>
+      <c r="D21" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>OE</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="inlineStr">
+        <is>
+          <t>17-Meghalaya</t>
+        </is>
+      </c>
+      <c r="C22" s="0" t="n"/>
+      <c r="D22" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" s="0" t="n">
+        <v>152.43</v>
+      </c>
+      <c r="F22" s="0" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2784,7 +2963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelRow="0"/>
   <cols>
     <col width="39.5703125" customWidth="1" min="1" max="1"/>
@@ -2921,32 +3100,94 @@
       </c>
       <c r="B5" s="63" t="inlineStr">
         <is>
+          <t>07AARCM9332R1CQ</t>
+        </is>
+      </c>
+      <c r="C5" s="64" t="inlineStr">
+        <is>
+          <t>meesho</t>
+        </is>
+      </c>
+      <c r="D5" s="55" t="n">
+        <v>2406.8</v>
+      </c>
+      <c r="E5" s="55" t="n">
+        <v>56.71</v>
+      </c>
+      <c r="F5" s="55" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="G5" s="55" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="H5" s="55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" ht="15.75" customHeight="1" s="81">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>Liable to collect tax u/s 52(TCS)</t>
+        </is>
+      </c>
+      <c r="B6" s="65" t="inlineStr">
+        <is>
+          <t>07AAICA3918J1CV</t>
+        </is>
+      </c>
+      <c r="C6" s="64" t="inlineStr">
+        <is>
+          <t>amazon</t>
+        </is>
+      </c>
+      <c r="D6" s="55" t="n">
+        <v>193.2</v>
+      </c>
+      <c r="E6" s="55" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="F6" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="55" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="15.75" customHeight="1" s="81">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>Liable to collect tax u/s 52(TCS)</t>
+        </is>
+      </c>
+      <c r="B7" s="63" t="inlineStr">
+        <is>
           <t>07AACCF0683K1CU</t>
         </is>
       </c>
-      <c r="C5" s="64" t="inlineStr">
+      <c r="C7" s="64" t="inlineStr">
         <is>
           <t>flipkart</t>
         </is>
       </c>
-      <c r="D5" s="55" t="n">
+      <c r="D7" s="55" t="n">
         <v>1127.19</v>
       </c>
-      <c r="E5" s="55" t="n">
+      <c r="E7" s="55" t="n">
         <v>33.81</v>
       </c>
-      <c r="F5" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="55" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="55" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" ht="15.75" customHeight="1" s="81"/>
-    <row r="7" ht="15.75" customHeight="1" s="81"/>
+      <c r="F7" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="55" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="55" t="n">
+        <v>0</v>
+      </c>
+    </row>
     <row r="8" ht="15.75" customHeight="1" s="81"/>
   </sheetData>
   <dataValidations count="39">

</xml_diff>

<commit_message>
May 20, 2026, 7:24 PM
</commit_message>
<xml_diff>
--- a/storage/exports/4/07TCRPS8655B1ZK/022026/gstr1.xlsx
+++ b/storage/exports/4/07TCRPS8655B1ZK/022026/gstr1.xlsx
@@ -1299,7 +1299,7 @@
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>RAT6SO2600000021</t>
+          <t>RAT6SO2600000022</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -1308,7 +1308,7 @@
         </is>
       </c>
       <c r="D9" s="0" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E9" s="0" t="n">
         <v>0</v>
@@ -1520,7 +1520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelRow="0"/>
   <cols>
     <col width="22.42578125" customWidth="1" min="1" max="1"/>
@@ -1668,7 +1668,7 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>18-Assam</t>
+          <t>10-Bihar</t>
         </is>
       </c>
       <c r="C7" s="0" t="n"/>
@@ -1676,7 +1676,7 @@
         <v>3</v>
       </c>
       <c r="E7" s="0" t="n">
-        <v>0</v>
+        <v>264.07</v>
       </c>
       <c r="F7" s="0" t="n">
         <v>0</v>
@@ -1690,7 +1690,7 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>10-Bihar</t>
+          <t>07-Delhi</t>
         </is>
       </c>
       <c r="C8" s="0" t="n"/>
@@ -1698,7 +1698,7 @@
         <v>3</v>
       </c>
       <c r="E8" s="0" t="n">
-        <v>264.07</v>
+        <v>516.5</v>
       </c>
       <c r="F8" s="0" t="n">
         <v>0</v>
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>04-Chandigarh</t>
+          <t>24-Gujarat</t>
         </is>
       </c>
       <c r="C9" s="0" t="n"/>
@@ -1720,7 +1720,7 @@
         <v>3</v>
       </c>
       <c r="E9" s="0" t="n">
-        <v>0</v>
+        <v>219.42</v>
       </c>
       <c r="F9" s="0" t="n">
         <v>0</v>
@@ -1734,7 +1734,7 @@
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>07-Delhi</t>
+          <t>02-Himachal Pradesh</t>
         </is>
       </c>
       <c r="C10" s="0" t="n"/>
@@ -1742,7 +1742,7 @@
         <v>3</v>
       </c>
       <c r="E10" s="0" t="n">
-        <v>516.5</v>
+        <v>200</v>
       </c>
       <c r="F10" s="0" t="n">
         <v>0</v>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>24-Gujarat</t>
+          <t>29-Karnataka</t>
         </is>
       </c>
       <c r="C11" s="0" t="n"/>
@@ -1764,7 +1764,7 @@
         <v>3</v>
       </c>
       <c r="E11" s="0" t="n">
-        <v>219.42</v>
+        <v>654.38</v>
       </c>
       <c r="F11" s="0" t="n">
         <v>0</v>
@@ -1778,7 +1778,7 @@
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>06-Haryana</t>
+          <t>27-Maharashtra</t>
         </is>
       </c>
       <c r="C12" s="0" t="n"/>
@@ -1786,7 +1786,7 @@
         <v>3</v>
       </c>
       <c r="E12" s="0" t="n">
-        <v>0</v>
+        <v>319.41</v>
       </c>
       <c r="F12" s="0" t="n">
         <v>0</v>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>02-Himachal Pradesh</t>
+          <t>21-Odisha</t>
         </is>
       </c>
       <c r="C13" s="0" t="n"/>
@@ -1808,7 +1808,7 @@
         <v>3</v>
       </c>
       <c r="E13" s="0" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="F13" s="0" t="n">
         <v>0</v>
@@ -1822,7 +1822,7 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>20-Jharkhand</t>
+          <t>03-Punjab</t>
         </is>
       </c>
       <c r="C14" s="0" t="n"/>
@@ -1830,7 +1830,7 @@
         <v>3</v>
       </c>
       <c r="E14" s="0" t="n">
-        <v>0</v>
+        <v>315.54</v>
       </c>
       <c r="F14" s="0" t="n">
         <v>0</v>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>29-Karnataka</t>
+          <t>08-Rajasthan</t>
         </is>
       </c>
       <c r="C15" s="0" t="n"/>
@@ -1852,7 +1852,7 @@
         <v>3</v>
       </c>
       <c r="E15" s="0" t="n">
-        <v>654.38</v>
+        <v>113.59</v>
       </c>
       <c r="F15" s="0" t="n">
         <v>0</v>
@@ -1866,7 +1866,7 @@
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>27-Maharashtra</t>
+          <t>33-Tamil Nadu</t>
         </is>
       </c>
       <c r="C16" s="0" t="n"/>
@@ -1874,7 +1874,7 @@
         <v>3</v>
       </c>
       <c r="E16" s="0" t="n">
-        <v>319.41</v>
+        <v>524.27</v>
       </c>
       <c r="F16" s="0" t="n">
         <v>0</v>
@@ -1888,7 +1888,7 @@
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>21-Odisha</t>
+          <t>36-Telangana</t>
         </is>
       </c>
       <c r="C17" s="0" t="n"/>
@@ -1896,7 +1896,7 @@
         <v>3</v>
       </c>
       <c r="E17" s="0" t="n">
-        <v>0</v>
+        <v>-348.54</v>
       </c>
       <c r="F17" s="0" t="n">
         <v>0</v>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>03-Punjab</t>
+          <t>09-Uttar Pradesh</t>
         </is>
       </c>
       <c r="C18" s="0" t="n"/>
@@ -1918,7 +1918,7 @@
         <v>3</v>
       </c>
       <c r="E18" s="0" t="n">
-        <v>315.54</v>
+        <v>114.56</v>
       </c>
       <c r="F18" s="0" t="n">
         <v>0</v>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>08-Rajasthan</t>
+          <t>19-West Bengal</t>
         </is>
       </c>
       <c r="C19" s="0" t="n"/>
@@ -1940,7 +1940,7 @@
         <v>3</v>
       </c>
       <c r="E19" s="0" t="n">
-        <v>113.59</v>
+        <v>0</v>
       </c>
       <c r="F19" s="0" t="n">
         <v>0</v>
@@ -1954,7 +1954,7 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>33-Tamil Nadu</t>
+          <t>17-Meghalaya</t>
         </is>
       </c>
       <c r="C20" s="0" t="n"/>
@@ -1962,53 +1962,9 @@
         <v>3</v>
       </c>
       <c r="E20" s="0" t="n">
-        <v>524.27</v>
+        <v>152.43</v>
       </c>
       <c r="F20" s="0" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="0" t="inlineStr">
-        <is>
-          <t>OE</t>
-        </is>
-      </c>
-      <c r="B21" s="0" t="inlineStr">
-        <is>
-          <t>19-West Bengal</t>
-        </is>
-      </c>
-      <c r="C21" s="0" t="n"/>
-      <c r="D21" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="E21" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="0" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="0" t="inlineStr">
-        <is>
-          <t>OE</t>
-        </is>
-      </c>
-      <c r="B22" s="0" t="inlineStr">
-        <is>
-          <t>17-Meghalaya</t>
-        </is>
-      </c>
-      <c r="C22" s="0" t="n"/>
-      <c r="D22" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="E22" s="0" t="n">
-        <v>152.43</v>
-      </c>
-      <c r="F22" s="0" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3173,10 +3129,10 @@
         </is>
       </c>
       <c r="D7" s="55" t="n">
-        <v>1127.19</v>
+        <v>1259.23</v>
       </c>
       <c r="E7" s="55" t="n">
-        <v>33.81</v>
+        <v>37.77</v>
       </c>
       <c r="F7" s="55" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
May 21, 2026, 3:02 PM
</commit_message>
<xml_diff>
--- a/storage/exports/4/07TCRPS8655B1ZK/022026/gstr1.xlsx
+++ b/storage/exports/4/07TCRPS8655B1ZK/022026/gstr1.xlsx
@@ -1276,16 +1276,16 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>FAWRLX2600000063</t>
+          <t>FAWRLX2600000076</t>
         </is>
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>FAWRLX2600000079</t>
+          <t>FAWRLX2600000081</t>
         </is>
       </c>
       <c r="D8" s="0" t="n">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="E8" s="0" t="n">
         <v>0</v>
@@ -1299,7 +1299,7 @@
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>RAT6SO2600000022</t>
+          <t>RAT6SO2600000024</t>
         </is>
       </c>
       <c r="C9" s="0" t="inlineStr">
@@ -1308,7 +1308,7 @@
         </is>
       </c>
       <c r="D9" s="0" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E9" s="0" t="n">
         <v>0</v>
@@ -1322,16 +1322,16 @@
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>CANQ1W2600000008</t>
+          <t>CANQ1W2600000011</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>CANQ1W2600000012</t>
+          <t>CANQ1W2600000013</t>
         </is>
       </c>
       <c r="D10" s="0" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E10" s="0" t="n">
         <v>0</v>
@@ -1632,7 +1632,7 @@
         <v>3</v>
       </c>
       <c r="E5" s="0" t="n">
-        <v>578.64</v>
+        <v>488.35</v>
       </c>
       <c r="F5" s="0" t="n">
         <v>0</v>
@@ -1646,7 +1646,7 @@
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>18-Assam</t>
+          <t>10-Bihar</t>
         </is>
       </c>
       <c r="C6" s="0" t="n"/>
@@ -1654,7 +1654,7 @@
         <v>3</v>
       </c>
       <c r="E6" s="0" t="n">
-        <v>234.95</v>
+        <v>0</v>
       </c>
       <c r="F6" s="0" t="n">
         <v>0</v>
@@ -1668,7 +1668,7 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>10-Bihar</t>
+          <t>07-Delhi</t>
         </is>
       </c>
       <c r="C7" s="0" t="n"/>
@@ -1676,7 +1676,7 @@
         <v>3</v>
       </c>
       <c r="E7" s="0" t="n">
-        <v>264.07</v>
+        <v>516.5</v>
       </c>
       <c r="F7" s="0" t="n">
         <v>0</v>
@@ -1690,7 +1690,7 @@
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>07-Delhi</t>
+          <t>24-Gujarat</t>
         </is>
       </c>
       <c r="C8" s="0" t="n"/>
@@ -1698,7 +1698,7 @@
         <v>3</v>
       </c>
       <c r="E8" s="0" t="n">
-        <v>516.5</v>
+        <v>219.42</v>
       </c>
       <c r="F8" s="0" t="n">
         <v>0</v>
@@ -1712,7 +1712,7 @@
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>24-Gujarat</t>
+          <t>02-Himachal Pradesh</t>
         </is>
       </c>
       <c r="C9" s="0" t="n"/>
@@ -1720,7 +1720,7 @@
         <v>3</v>
       </c>
       <c r="E9" s="0" t="n">
-        <v>219.42</v>
+        <v>200</v>
       </c>
       <c r="F9" s="0" t="n">
         <v>0</v>
@@ -1734,7 +1734,7 @@
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>02-Himachal Pradesh</t>
+          <t>20-Jharkhand</t>
         </is>
       </c>
       <c r="C10" s="0" t="n"/>
@@ -1742,7 +1742,7 @@
         <v>3</v>
       </c>
       <c r="E10" s="0" t="n">
-        <v>200</v>
+        <v>103.88</v>
       </c>
       <c r="F10" s="0" t="n">
         <v>0</v>
@@ -1764,7 +1764,7 @@
         <v>3</v>
       </c>
       <c r="E11" s="0" t="n">
-        <v>654.38</v>
+        <v>335.92</v>
       </c>
       <c r="F11" s="0" t="n">
         <v>0</v>
@@ -1786,7 +1786,7 @@
         <v>3</v>
       </c>
       <c r="E12" s="0" t="n">
-        <v>319.41</v>
+        <v>193.2</v>
       </c>
       <c r="F12" s="0" t="n">
         <v>0</v>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>21-Odisha</t>
+          <t>17-Meghalaya</t>
         </is>
       </c>
       <c r="C13" s="0" t="n"/>
@@ -1808,7 +1808,7 @@
         <v>3</v>
       </c>
       <c r="E13" s="0" t="n">
-        <v>0</v>
+        <v>152.43</v>
       </c>
       <c r="F13" s="0" t="n">
         <v>0</v>
@@ -1822,7 +1822,7 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>03-Punjab</t>
+          <t>21-Odisha</t>
         </is>
       </c>
       <c r="C14" s="0" t="n"/>
@@ -1830,7 +1830,7 @@
         <v>3</v>
       </c>
       <c r="E14" s="0" t="n">
-        <v>315.54</v>
+        <v>104.86</v>
       </c>
       <c r="F14" s="0" t="n">
         <v>0</v>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>08-Rajasthan</t>
+          <t>03-Punjab</t>
         </is>
       </c>
       <c r="C15" s="0" t="n"/>
@@ -1852,7 +1852,7 @@
         <v>3</v>
       </c>
       <c r="E15" s="0" t="n">
-        <v>113.59</v>
+        <v>315.54</v>
       </c>
       <c r="F15" s="0" t="n">
         <v>0</v>
@@ -1866,7 +1866,7 @@
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>33-Tamil Nadu</t>
+          <t>08-Rajasthan</t>
         </is>
       </c>
       <c r="C16" s="0" t="n"/>
@@ -1874,7 +1874,7 @@
         <v>3</v>
       </c>
       <c r="E16" s="0" t="n">
-        <v>524.27</v>
+        <v>113.59</v>
       </c>
       <c r="F16" s="0" t="n">
         <v>0</v>
@@ -1888,7 +1888,7 @@
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>36-Telangana</t>
+          <t>33-Tamil Nadu</t>
         </is>
       </c>
       <c r="C17" s="0" t="n"/>
@@ -1896,7 +1896,7 @@
         <v>3</v>
       </c>
       <c r="E17" s="0" t="n">
-        <v>-348.54</v>
+        <v>410.68</v>
       </c>
       <c r="F17" s="0" t="n">
         <v>0</v>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>09-Uttar Pradesh</t>
+          <t>36-Telangana</t>
         </is>
       </c>
       <c r="C18" s="0" t="n"/>
@@ -1918,7 +1918,7 @@
         <v>3</v>
       </c>
       <c r="E18" s="0" t="n">
-        <v>114.56</v>
+        <v>-348.54</v>
       </c>
       <c r="F18" s="0" t="n">
         <v>0</v>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>19-West Bengal</t>
+          <t>09-Uttar Pradesh</t>
         </is>
       </c>
       <c r="C19" s="0" t="n"/>
@@ -1940,7 +1940,7 @@
         <v>3</v>
       </c>
       <c r="E19" s="0" t="n">
-        <v>0</v>
+        <v>-11.65</v>
       </c>
       <c r="F19" s="0" t="n">
         <v>0</v>
@@ -1954,7 +1954,7 @@
       </c>
       <c r="B20" s="0" t="inlineStr">
         <is>
-          <t>17-Meghalaya</t>
+          <t>19-West Bengal</t>
         </is>
       </c>
       <c r="C20" s="0" t="n"/>
@@ -1962,7 +1962,7 @@
         <v>3</v>
       </c>
       <c r="E20" s="0" t="n">
-        <v>152.43</v>
+        <v>0</v>
       </c>
       <c r="F20" s="0" t="n">
         <v>0</v>
@@ -3129,10 +3129,10 @@
         </is>
       </c>
       <c r="D7" s="55" t="n">
-        <v>1259.23</v>
+        <v>194.19</v>
       </c>
       <c r="E7" s="55" t="n">
-        <v>37.77</v>
+        <v>5.81</v>
       </c>
       <c r="F7" s="55" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
May 21, 2026, 3:41 PM
</commit_message>
<xml_diff>
--- a/storage/exports/4/07TCRPS8655B1ZK/022026/gstr1.xlsx
+++ b/storage/exports/4/07TCRPS8655B1ZK/022026/gstr1.xlsx
@@ -1281,11 +1281,11 @@
       </c>
       <c r="C8" s="0" t="inlineStr">
         <is>
-          <t>FAWRLX2600000081</t>
+          <t>FAWRLX2600000079</t>
         </is>
       </c>
       <c r="D8" s="0" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E8" s="0" t="n">
         <v>0</v>
@@ -1327,11 +1327,11 @@
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>CANQ1W2600000013</t>
+          <t>CANQ1W2600000012</t>
         </is>
       </c>
       <c r="D10" s="0" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E10" s="0" t="n">
         <v>0</v>
@@ -1520,7 +1520,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelRow="0"/>
   <cols>
     <col width="22.42578125" customWidth="1" min="1" max="1"/>
@@ -1734,7 +1734,7 @@
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>20-Jharkhand</t>
+          <t>29-Karnataka</t>
         </is>
       </c>
       <c r="C10" s="0" t="n"/>
@@ -1742,7 +1742,7 @@
         <v>3</v>
       </c>
       <c r="E10" s="0" t="n">
-        <v>103.88</v>
+        <v>335.92</v>
       </c>
       <c r="F10" s="0" t="n">
         <v>0</v>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>29-Karnataka</t>
+          <t>27-Maharashtra</t>
         </is>
       </c>
       <c r="C11" s="0" t="n"/>
@@ -1764,7 +1764,7 @@
         <v>3</v>
       </c>
       <c r="E11" s="0" t="n">
-        <v>335.92</v>
+        <v>193.2</v>
       </c>
       <c r="F11" s="0" t="n">
         <v>0</v>
@@ -1778,7 +1778,7 @@
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>27-Maharashtra</t>
+          <t>17-Meghalaya</t>
         </is>
       </c>
       <c r="C12" s="0" t="n"/>
@@ -1786,7 +1786,7 @@
         <v>3</v>
       </c>
       <c r="E12" s="0" t="n">
-        <v>193.2</v>
+        <v>152.43</v>
       </c>
       <c r="F12" s="0" t="n">
         <v>0</v>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>17-Meghalaya</t>
+          <t>21-Odisha</t>
         </is>
       </c>
       <c r="C13" s="0" t="n"/>
@@ -1808,7 +1808,7 @@
         <v>3</v>
       </c>
       <c r="E13" s="0" t="n">
-        <v>152.43</v>
+        <v>0</v>
       </c>
       <c r="F13" s="0" t="n">
         <v>0</v>
@@ -1822,7 +1822,7 @@
       </c>
       <c r="B14" s="0" t="inlineStr">
         <is>
-          <t>21-Odisha</t>
+          <t>03-Punjab</t>
         </is>
       </c>
       <c r="C14" s="0" t="n"/>
@@ -1830,7 +1830,7 @@
         <v>3</v>
       </c>
       <c r="E14" s="0" t="n">
-        <v>104.86</v>
+        <v>315.54</v>
       </c>
       <c r="F14" s="0" t="n">
         <v>0</v>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="B15" s="0" t="inlineStr">
         <is>
-          <t>03-Punjab</t>
+          <t>08-Rajasthan</t>
         </is>
       </c>
       <c r="C15" s="0" t="n"/>
@@ -1852,7 +1852,7 @@
         <v>3</v>
       </c>
       <c r="E15" s="0" t="n">
-        <v>315.54</v>
+        <v>113.59</v>
       </c>
       <c r="F15" s="0" t="n">
         <v>0</v>
@@ -1866,7 +1866,7 @@
       </c>
       <c r="B16" s="0" t="inlineStr">
         <is>
-          <t>08-Rajasthan</t>
+          <t>33-Tamil Nadu</t>
         </is>
       </c>
       <c r="C16" s="0" t="n"/>
@@ -1874,7 +1874,7 @@
         <v>3</v>
       </c>
       <c r="E16" s="0" t="n">
-        <v>113.59</v>
+        <v>410.68</v>
       </c>
       <c r="F16" s="0" t="n">
         <v>0</v>
@@ -1888,7 +1888,7 @@
       </c>
       <c r="B17" s="0" t="inlineStr">
         <is>
-          <t>33-Tamil Nadu</t>
+          <t>36-Telangana</t>
         </is>
       </c>
       <c r="C17" s="0" t="n"/>
@@ -1896,7 +1896,7 @@
         <v>3</v>
       </c>
       <c r="E17" s="0" t="n">
-        <v>410.68</v>
+        <v>-348.54</v>
       </c>
       <c r="F17" s="0" t="n">
         <v>0</v>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="B18" s="0" t="inlineStr">
         <is>
-          <t>36-Telangana</t>
+          <t>09-Uttar Pradesh</t>
         </is>
       </c>
       <c r="C18" s="0" t="n"/>
@@ -1918,7 +1918,7 @@
         <v>3</v>
       </c>
       <c r="E18" s="0" t="n">
-        <v>-348.54</v>
+        <v>-11.65</v>
       </c>
       <c r="F18" s="0" t="n">
         <v>0</v>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="B19" s="0" t="inlineStr">
         <is>
-          <t>09-Uttar Pradesh</t>
+          <t>19-West Bengal</t>
         </is>
       </c>
       <c r="C19" s="0" t="n"/>
@@ -1940,31 +1940,9 @@
         <v>3</v>
       </c>
       <c r="E19" s="0" t="n">
-        <v>-11.65</v>
+        <v>0</v>
       </c>
       <c r="F19" s="0" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="0" t="inlineStr">
-        <is>
-          <t>OE</t>
-        </is>
-      </c>
-      <c r="B20" s="0" t="inlineStr">
-        <is>
-          <t>19-West Bengal</t>
-        </is>
-      </c>
-      <c r="C20" s="0" t="n"/>
-      <c r="D20" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="E20" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" s="0" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3129,10 +3107,10 @@
         </is>
       </c>
       <c r="D7" s="55" t="n">
-        <v>194.19</v>
+        <v>-14.55</v>
       </c>
       <c r="E7" s="55" t="n">
-        <v>5.81</v>
+        <v>-0.45</v>
       </c>
       <c r="F7" s="55" t="n">
         <v>0</v>

</xml_diff>